<commit_message>
data upload to queue
</commit_message>
<xml_diff>
--- a/Data/IJ_Config.xlsx
+++ b/Data/IJ_Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\UiPath\IJ_WysylanieFaktur\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5991767-CE53-4180-AE9F-23A1E9D6BE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12F85B9-6A70-49A2-9EDE-CB3DE7B6034E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
   <si>
     <t>Name</t>
   </si>
@@ -175,6 +175,18 @@
   </si>
   <si>
     <t>NUMER FAKTURY</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>https://funnyjudowarszawa.fakturownia.pl</t>
+  </si>
+  <si>
+    <t>ColumnKontakt</t>
+  </si>
+  <si>
+    <t>KONTAKT</t>
   </si>
 </sst>
 </file>
@@ -540,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z994"/>
+  <dimension ref="A1:Z995"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -639,9 +651,23 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+    </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1625,6 +1651,7 @@
     <row r="992" ht="14.25" customHeight="1"/>
     <row r="993" ht="14.25" customHeight="1"/>
     <row r="994" ht="14.25" customHeight="1"/>
+    <row r="995" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>